<commit_message>
Add R&D capitalization, employee count, and fix golden eval
- compute.py: R&D amortization/asset/OI adjustment (20-quarter schedule
  using 3 prior annual + 12 quarterly actuals) and employee count from
  10-K HTML parsing
- eval.py: now evaluates all 28 fields per quarter including R&D and
  employee count
- Fix golden_eval.xlsx: corrected FY2025 Q4 R&D from 6,434M to 3,714M
  (formula was missing Q1 subtraction)
- Result: 336/336 fields, 0 mismatches, 0 missing

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8741E6A-F7FD-D544-8D0F-ED225019D733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{3488ECCA-FDB0-5644-8569-5388F9B2B4CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="3080" windowWidth="27240" windowHeight="16760" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
+    <workbookView xWindow="6300" yWindow="2880" windowWidth="27240" windowHeight="16760" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
   <sheets>
     <sheet name="manual_audit_entry_v1" sheetId="1" r:id="rId1"/>
@@ -3846,13 +3846,13 @@
         <v>-61000000</v>
       </c>
       <c r="AS9" s="3">
-        <v>2042000000</v>
+        <v>1906000000</v>
       </c>
       <c r="AT9" s="3">
-        <v>27143125000</v>
+        <v>24423125000</v>
       </c>
       <c r="AU9" s="3">
-        <v>4392000000</v>
+        <v>1808000000</v>
       </c>
       <c r="AV9" s="3" t="s">
         <v>473</v>
@@ -3994,13 +3994,13 @@
         <v>-63000000</v>
       </c>
       <c r="AS10" s="3">
-        <v>2192400000</v>
+        <v>2056400000</v>
       </c>
       <c r="AT10" s="3">
-        <v>29090125000</v>
+        <v>26506125000</v>
       </c>
       <c r="AU10" s="3">
-        <v>1796600000</v>
+        <v>1932600000</v>
       </c>
       <c r="AV10" s="3" t="s">
         <v>473</v>
@@ -4142,13 +4142,13 @@
         <v>-62000000</v>
       </c>
       <c r="AS11" s="3">
-        <v>2357900000</v>
+        <v>2221900000</v>
       </c>
       <c r="AT11" s="3">
-        <v>31188725000</v>
+        <v>28740725000</v>
       </c>
       <c r="AU11" s="3">
-        <v>1933100000</v>
+        <v>2069100000</v>
       </c>
       <c r="AV11" s="3" t="s">
         <v>473</v>
@@ -4290,13 +4290,13 @@
         <v>-61000000</v>
       </c>
       <c r="AS12" s="3">
-        <v>2544100000</v>
+        <v>2408100000</v>
       </c>
       <c r="AT12" s="3">
-        <v>33535825000</v>
+        <v>31223825000</v>
       </c>
       <c r="AU12" s="3">
-        <v>2160900000</v>
+        <v>2296900000</v>
       </c>
       <c r="AV12" s="3" t="s">
         <v>473</v>
@@ -4441,13 +4441,13 @@
         <v>-73000000</v>
       </c>
       <c r="AS13" s="3">
-        <v>2770650000</v>
+        <v>2634650000</v>
       </c>
       <c r="AT13" s="3">
-        <v>36503725000</v>
+        <v>34327725000</v>
       </c>
       <c r="AU13" s="3">
-        <v>2741350000</v>
+        <v>2877350000</v>
       </c>
       <c r="AV13" s="3" t="s">
         <v>473</v>
@@ -38876,11 +38876,11 @@
         <v>20</v>
       </c>
       <c r="G12" s="4">
-        <v>6434000000</v>
+        <v>3714000000</v>
       </c>
       <c r="I12" s="20">
         <f t="shared" si="0"/>
-        <v>6434000000</v>
+        <v>3714000000</v>
       </c>
       <c r="J12" s="20">
         <f t="shared" si="2"/>
@@ -38960,15 +38960,15 @@
       </c>
       <c r="AD12" s="21">
         <f t="shared" si="6"/>
-        <v>2042000000</v>
+        <v>1906000000</v>
       </c>
       <c r="AE12" s="21">
         <f t="shared" si="3"/>
-        <v>27143125000</v>
+        <v>24423125000</v>
       </c>
       <c r="AF12" s="21">
         <f t="shared" si="1"/>
-        <v>4392000000</v>
+        <v>1808000000</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.2">
@@ -39003,7 +39003,7 @@
       </c>
       <c r="J13" s="20">
         <f t="shared" si="2"/>
-        <v>6434000000</v>
+        <v>3714000000</v>
       </c>
       <c r="K13" s="20">
         <f t="shared" si="5"/>
@@ -39079,15 +39079,15 @@
       </c>
       <c r="AD13" s="21">
         <f t="shared" si="6"/>
-        <v>2192400000</v>
+        <v>2056400000</v>
       </c>
       <c r="AE13" s="21">
         <f t="shared" si="3"/>
-        <v>29090125000</v>
+        <v>26506125000</v>
       </c>
       <c r="AF13" s="21">
         <f t="shared" si="1"/>
-        <v>1796600000</v>
+        <v>1932600000</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.2">
@@ -39126,7 +39126,7 @@
       </c>
       <c r="K14" s="20">
         <f t="shared" si="5"/>
-        <v>6434000000</v>
+        <v>3714000000</v>
       </c>
       <c r="L14" s="20">
         <f t="shared" si="7"/>
@@ -39198,15 +39198,15 @@
       </c>
       <c r="AD14" s="21">
         <f t="shared" si="6"/>
-        <v>2357900000</v>
+        <v>2221900000</v>
       </c>
       <c r="AE14" s="21">
         <f t="shared" si="3"/>
-        <v>31188725000</v>
+        <v>28740725000</v>
       </c>
       <c r="AF14" s="21">
         <f t="shared" si="1"/>
-        <v>1933100000</v>
+        <v>2069100000</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.2">
@@ -39249,7 +39249,7 @@
       </c>
       <c r="L15" s="20">
         <f t="shared" si="7"/>
-        <v>6434000000</v>
+        <v>3714000000</v>
       </c>
       <c r="M15" s="20">
         <f t="shared" si="8"/>
@@ -39317,15 +39317,15 @@
       </c>
       <c r="AD15" s="21">
         <f t="shared" si="6"/>
-        <v>2544100000</v>
+        <v>2408100000</v>
       </c>
       <c r="AE15" s="21">
         <f t="shared" si="3"/>
-        <v>33535825000</v>
+        <v>31223825000</v>
       </c>
       <c r="AF15" s="21">
         <f t="shared" si="1"/>
-        <v>2160900000</v>
+        <v>2296900000</v>
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.2">
@@ -39372,7 +39372,7 @@
       </c>
       <c r="M16" s="20">
         <f t="shared" si="8"/>
-        <v>6434000000</v>
+        <v>3714000000</v>
       </c>
       <c r="N16" s="20">
         <f t="shared" si="9"/>
@@ -39436,15 +39436,15 @@
       </c>
       <c r="AD16" s="21">
         <f t="shared" si="6"/>
-        <v>2770650000</v>
+        <v>2634650000</v>
       </c>
       <c r="AE16" s="21">
         <f t="shared" si="3"/>
-        <v>36503725000</v>
+        <v>34327725000</v>
       </c>
       <c r="AF16" s="21">
         <f t="shared" si="1"/>
-        <v>2741350000</v>
+        <v>2877350000</v>
       </c>
     </row>
     <row r="17" spans="1:32" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Fix restatement scoping, equity/net income concepts, and eval threshold
extract.py:
- Restatement overrides now apply to all component types (stock, flow,
  per_period), not just flow. Scoped to filings with
  DocumentFinStmtErrorCorrectionFlag=true or amended form types only.
- Stock split detection from StockholdersEquityNoteStockSplitConversionRatio1
  prevents pre-split diluted share overrides.
- equity_q prefers StockholdersEquityIncludingPortionAttributableToNoncontrollingInterest
  (matches NOPAT basis for ROIC).
- net_income_q prefers ProfitLoss (consolidated, ties to CFO for accruals ratio).

eval.py: Tighten close-match threshold from 1% to 0.1%. The old threshold
hid real errors (NCI discrepancies) behind false "close" matches.

NVDA: 336/336, 0 mismatches. DELL: 5 mismatches remaining (all FY2025 Q4
derivation from restated FY vs pre-restatement 9M YTD).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{3488ECCA-FDB0-5644-8569-5388F9B2B4CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{4AF6F0BA-11B6-0A42-BEBB-4B4642CA6D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6300" yWindow="2880" windowWidth="27240" windowHeight="16760" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
+    <workbookView xWindow="41100" yWindow="1680" windowWidth="27240" windowHeight="16760" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
   <sheets>
     <sheet name="manual_audit_entry_v1" sheetId="1" r:id="rId1"/>
@@ -2498,6 +2498,8 @@
     <col min="48" max="48" width="29.6640625" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="22.83203125" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="13.83203125" customWidth="1"/>
     <col min="59" max="59" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7305,7 +7307,7 @@
       <c r="BA32" s="3"/>
       <c r="BB32" s="3"/>
     </row>
-    <row r="33" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>3</v>
       </c>
@@ -7456,7 +7458,7 @@
       <c r="BA33" s="3"/>
       <c r="BB33" s="3"/>
     </row>
-    <row r="34" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>3</v>
       </c>
@@ -7607,7 +7609,7 @@
       <c r="BA34" s="3"/>
       <c r="BB34" s="3"/>
     </row>
-    <row r="35" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>3</v>
       </c>
@@ -7758,7 +7760,7 @@
       <c r="BA35" s="3"/>
       <c r="BB35" s="3"/>
     </row>
-    <row r="36" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>3</v>
       </c>
@@ -7906,10 +7908,8 @@
       <c r="AW36" s="7">
         <v>2000</v>
       </c>
-      <c r="BA36" s="3"/>
-      <c r="BB36" s="3"/>
     </row>
-    <row r="37" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>3</v>
       </c>
@@ -8057,10 +8057,9 @@
       <c r="AW37" s="7">
         <v>2000</v>
       </c>
-      <c r="BA37" s="3"/>
       <c r="BB37" s="3"/>
     </row>
-    <row r="38" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>4</v>
       </c>
@@ -8208,11 +8207,11 @@
       <c r="AW38" s="7">
         <v>133000</v>
       </c>
-      <c r="AY38" s="3"/>
-      <c r="BA38" s="3"/>
+      <c r="AY38" s="2"/>
       <c r="BB38" s="3"/>
+      <c r="BC38" s="3"/>
     </row>
-    <row r="39" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>4</v>
       </c>
@@ -8360,11 +8359,11 @@
       <c r="AW39" s="7">
         <v>133000</v>
       </c>
-      <c r="AY39" s="3"/>
-      <c r="BA39" s="3"/>
+      <c r="AY39" s="2"/>
       <c r="BB39" s="3"/>
+      <c r="BC39" s="3"/>
     </row>
-    <row r="40" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>4</v>
       </c>
@@ -8512,11 +8511,11 @@
       <c r="AW40" s="7">
         <v>133000</v>
       </c>
-      <c r="AY40" s="3"/>
-      <c r="BA40" s="3"/>
+      <c r="AY40" s="2"/>
       <c r="BB40" s="3"/>
+      <c r="BC40" s="3"/>
     </row>
-    <row r="41" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>4</v>
       </c>
@@ -8596,7 +8595,7 @@
         <v>1344000000</v>
       </c>
       <c r="AA41" s="9">
-        <v>-2309000000</v>
+        <v>-2132000000</v>
       </c>
       <c r="AB41">
         <v>6982000000</v>
@@ -8632,13 +8631,13 @@
         <v>3622000000</v>
       </c>
       <c r="AM41">
-        <v>19389000000</v>
+        <v>19226000000</v>
       </c>
       <c r="AN41">
         <v>1208000000</v>
       </c>
       <c r="AO41">
-        <v>82089000000</v>
+        <v>82126000000</v>
       </c>
       <c r="AP41">
         <v>203000000</v>
@@ -8664,11 +8663,11 @@
       <c r="AW41">
         <v>120000</v>
       </c>
-      <c r="AY41" s="3"/>
-      <c r="BA41" s="3"/>
+      <c r="AY41" s="2"/>
       <c r="BB41" s="3"/>
+      <c r="BC41" s="3"/>
     </row>
-    <row r="42" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>4</v>
       </c>
@@ -8816,11 +8815,11 @@
       <c r="AW42">
         <v>120000</v>
       </c>
-      <c r="AY42" s="3"/>
-      <c r="BA42" s="3"/>
+      <c r="AY42" s="2"/>
       <c r="BB42" s="3"/>
+      <c r="BC42" s="3"/>
     </row>
-    <row r="43" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>4</v>
       </c>
@@ -8968,11 +8967,11 @@
       <c r="AW43">
         <v>120000</v>
       </c>
-      <c r="AY43" s="3"/>
-      <c r="BA43" s="3"/>
+      <c r="AY43" s="2"/>
       <c r="BB43" s="3"/>
+      <c r="BC43" s="3"/>
     </row>
-    <row r="44" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>4</v>
       </c>
@@ -9120,11 +9119,11 @@
       <c r="AW44">
         <v>120000</v>
       </c>
-      <c r="AY44" s="3"/>
-      <c r="BA44" s="3"/>
+      <c r="AY44" s="2"/>
       <c r="BB44" s="3"/>
+      <c r="BC44" s="3"/>
     </row>
-    <row r="45" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>4</v>
       </c>
@@ -9272,11 +9271,11 @@
       <c r="AW45">
         <v>108000</v>
       </c>
-      <c r="AY45" s="3"/>
-      <c r="BA45" s="3"/>
+      <c r="AY45" s="2"/>
       <c r="BB45" s="3"/>
+      <c r="BC45" s="3"/>
     </row>
-    <row r="46" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>4</v>
       </c>
@@ -9424,11 +9423,9 @@
       <c r="AW46">
         <v>108000</v>
       </c>
-      <c r="AY46" s="3"/>
-      <c r="BA46" s="3"/>
       <c r="BB46" s="3"/>
     </row>
-    <row r="47" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>4</v>
       </c>
@@ -9576,11 +9573,9 @@
       <c r="AW47">
         <v>108000</v>
       </c>
-      <c r="AY47" s="3"/>
-      <c r="BA47" s="3"/>
       <c r="BB47" s="3"/>
     </row>
-    <row r="48" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>4</v>
       </c>
@@ -9728,8 +9723,6 @@
       <c r="AW48">
         <v>108000</v>
       </c>
-      <c r="AY48" s="3"/>
-      <c r="BA48" s="3"/>
       <c r="BB48" s="3"/>
     </row>
     <row r="49" spans="1:77" x14ac:dyDescent="0.2">
@@ -9880,8 +9873,6 @@
       <c r="AW49">
         <v>97000</v>
       </c>
-      <c r="AY49" s="3"/>
-      <c r="BA49" s="3"/>
       <c r="BB49" s="3"/>
     </row>
     <row r="50" spans="1:77" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Sum current + noncurrent for operating lease liabilities, consolidate docs
Changed operating_lease_liabilities_q to sum OperatingLeaseLiabilityCurrent +
OperatingLeaseLiabilityNoncurrent instead of looking for the single total
concept. Fixes PLTR (which only tags the split) and handles restatement
overrides correctly for summed concepts. Merged extract_master_design.md
into extraction_logic.md and deleted the redundant file.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{4AF6F0BA-11B6-0A42-BEBB-4B4642CA6D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{73E64355-BA4F-E742-B06B-1A179AAA3869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41100" yWindow="1680" windowWidth="27240" windowHeight="16760" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
+    <workbookView xWindow="4640" yWindow="3120" windowWidth="27240" windowHeight="16760" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
   <sheets>
     <sheet name="manual_audit_entry_v1" sheetId="1" r:id="rId1"/>
@@ -3752,7 +3752,7 @@
         <v>8</v>
       </c>
       <c r="L9" s="2" t="d">
-        <v>2024-10-30</v>
+        <v>2024-10-28</v>
       </c>
       <c r="M9" s="2" t="d">
         <v>2025-01-26</v>

</xml_diff>

<commit_message>
Add PANW golden eval JSON, fix D&A Q3 2023 in spreadsheet
PANW: 336/336 exact matches, 0 mismatches.
All four companies now at 0 mismatches:
- NVDA: 303 exact + 33 close (Q4 rounding)
- DELL: 336/336 exact
- PLTR: 336/336 exact
- PANW: 336/336 exact

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{BECECC5B-E661-A044-91CB-723D672566B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{20D947B6-7498-C54F-9CDB-34B3479A46BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="600" windowWidth="37280" windowHeight="19080" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
@@ -11827,7 +11827,7 @@
         <v>-31199999.999999981</v>
       </c>
       <c r="AI62">
-        <v>142399999.99999991</v>
+        <v>155400000</v>
       </c>
       <c r="AJ62">
         <v>-18900000.000000007</v>
@@ -12687,6 +12687,10 @@
       <c r="AW67">
         <v>15289</v>
       </c>
+      <c r="BA67">
+        <f>70.7+97+1.8+1.7</f>
+        <v>171.2</v>
+      </c>
       <c r="BB67" s="3"/>
       <c r="BD67" s="3"/>
       <c r="BV67">
@@ -12849,7 +12853,10 @@
       <c r="AW68">
         <v>15289</v>
       </c>
-      <c r="BA68" s="3"/>
+      <c r="BA68" s="3">
+        <f>140.6+196+3.5-14.3-BA67</f>
+        <v>154.60000000000002</v>
+      </c>
       <c r="BB68" s="3"/>
       <c r="BV68">
         <v>2025</v>
@@ -13011,8 +13018,14 @@
       <c r="AW69">
         <v>15289</v>
       </c>
-      <c r="BA69" s="3"/>
-      <c r="BB69" s="3"/>
+      <c r="BA69" s="3">
+        <f>212.9+297.4+5.3-34.4-BA68-BA67</f>
+        <v>155.39999999999992</v>
+      </c>
+      <c r="BB69" s="3">
+        <f>+BA69*1000000</f>
+        <v>155399999.99999991</v>
+      </c>
       <c r="BV69">
         <v>2025</v>
       </c>

</xml_diff>

<commit_message>
Add UNP: 480/480 exact, no company-specific script needed
Union Pacific (UNP) passes all 28 fields across 20 quarters with zero
mismatches. First company added without requiring a companies/{ticker}.py
override — all fixes were master extractor improvements that benefit
future companies:
- FY context classification using DEI fiscal year dates
- Debt concepts for companies bundling debt with capital leases
- MaterialsSuppliesAndOther for railroad inventory
- Depreciation as standalone D&A concept
- HeldToMaturitySecuritiesCurrent for short-term investments
- HTML entity decoding in employee count parser

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{20D947B6-7498-C54F-9CDB-34B3479A46BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{CFB55B6D-8CF4-F147-B1BB-F351F3B45E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="600" windowWidth="37280" windowHeight="19080" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
@@ -13760,7 +13760,7 @@
         <v>0</v>
       </c>
       <c r="Y74">
-        <v>-512000000</v>
+        <v>512000000</v>
       </c>
       <c r="Z74">
         <v>2142000000</v>
@@ -13802,7 +13802,7 @@
         <v>728000000</v>
       </c>
       <c r="AM74">
-        <v>3617000000</v>
+        <v>952000000</v>
       </c>
       <c r="AN74">
         <v>1630000000</v>
@@ -13811,7 +13811,7 @@
         <v>65968000000</v>
       </c>
       <c r="AP74">
-        <v>0</v>
+        <v>28000000</v>
       </c>
       <c r="AQ74">
         <v>611500000</v>
@@ -13903,7 +13903,7 @@
         <v>0</v>
       </c>
       <c r="Y75">
-        <v>-389000000</v>
+        <v>389000000</v>
       </c>
       <c r="Z75">
         <v>1958000000</v>
@@ -13945,7 +13945,7 @@
         <v>742000000</v>
       </c>
       <c r="AM75">
-        <v>3504000000</v>
+        <v>894000000</v>
       </c>
       <c r="AN75">
         <v>1569000000</v>
@@ -13954,7 +13954,7 @@
         <v>66033000000</v>
       </c>
       <c r="AP75">
-        <v>0</v>
+        <v>24000000</v>
       </c>
       <c r="AQ75">
         <v>609500000</v>
@@ -14046,7 +14046,7 @@
         <v>0</v>
       </c>
       <c r="Y76">
-        <v>-421000000</v>
+        <v>421000000</v>
       </c>
       <c r="Z76">
         <v>1949000000</v>
@@ -14088,7 +14088,7 @@
         <v>770000000</v>
       </c>
       <c r="AM76">
-        <v>3580000000</v>
+        <v>936000000</v>
       </c>
       <c r="AN76">
         <v>1528000000</v>
@@ -14097,7 +14097,7 @@
         <v>66540000000</v>
       </c>
       <c r="AP76">
-        <v>0</v>
+        <v>32000000</v>
       </c>
       <c r="AQ76">
         <v>609800000</v>
@@ -14189,7 +14189,7 @@
         <v>0</v>
       </c>
       <c r="Y77">
-        <v>-532000000</v>
+        <v>532000000</v>
       </c>
       <c r="Z77">
         <v>2184000000</v>
@@ -14231,7 +14231,7 @@
         <v>743000000</v>
       </c>
       <c r="AM77">
-        <v>3683000000</v>
+        <v>856000000</v>
       </c>
       <c r="AN77">
         <v>1652000000</v>
@@ -14240,7 +14240,7 @@
         <v>67132000000</v>
       </c>
       <c r="AP77">
-        <v>0</v>
+        <v>23000000</v>
       </c>
       <c r="AQ77">
         <v>610200000</v>
@@ -14332,7 +14332,7 @@
         <v>0</v>
       </c>
       <c r="Y78">
-        <v>-499000000</v>
+        <v>499000000</v>
       </c>
       <c r="Z78">
         <v>2140000000</v>
@@ -14347,7 +14347,7 @@
         <v>31195000000</v>
       </c>
       <c r="AD78">
-        <v>1016000000</v>
+        <v>1338000000</v>
       </c>
       <c r="AE78">
         <v>925000000</v>
@@ -14374,7 +14374,7 @@
         <v>770000000</v>
       </c>
       <c r="AM78">
-        <v>3801000000</v>
+        <v>814000000</v>
       </c>
       <c r="AN78">
         <v>1641000000</v>
@@ -14383,7 +14383,7 @@
         <v>67266000000</v>
       </c>
       <c r="AP78">
-        <v>0</v>
+        <v>26000000</v>
       </c>
       <c r="AQ78">
         <v>610200000</v>
@@ -14475,7 +14475,7 @@
         <v>0</v>
       </c>
       <c r="Y79">
-        <v>-511000000</v>
+        <v>511000000</v>
       </c>
       <c r="Z79">
         <v>2184000000</v>
@@ -14490,7 +14490,7 @@
         <v>31165000000</v>
       </c>
       <c r="AD79">
-        <v>1722000000</v>
+        <v>1305000000</v>
       </c>
       <c r="AE79">
         <v>1137000000</v>
@@ -14517,7 +14517,7 @@
         <v>807000000</v>
       </c>
       <c r="AM79">
-        <v>3560000000</v>
+        <v>870000000</v>
       </c>
       <c r="AN79">
         <v>1673000000</v>
@@ -14526,7 +14526,7 @@
         <v>67817000000</v>
       </c>
       <c r="AP79">
-        <v>0</v>
+        <v>28000000</v>
       </c>
       <c r="AQ79">
         <v>610300000</v>
@@ -14618,7 +14618,7 @@
         <v>0</v>
       </c>
       <c r="Y80">
-        <v>-518000000</v>
+        <v>518000000</v>
       </c>
       <c r="Z80">
         <v>2189000000</v>
@@ -14633,7 +14633,7 @@
         <v>29761000000</v>
       </c>
       <c r="AD80">
-        <v>1726000000</v>
+        <v>1283000000</v>
       </c>
       <c r="AE80">
         <v>947000000</v>
@@ -14660,7 +14660,7 @@
         <v>775000000</v>
       </c>
       <c r="AM80">
-        <v>3714000000</v>
+        <v>830000000</v>
       </c>
       <c r="AN80">
         <v>1671000000</v>
@@ -14669,7 +14669,7 @@
         <v>67570000000</v>
       </c>
       <c r="AP80">
-        <v>0</v>
+        <v>33000000</v>
       </c>
       <c r="AQ80">
         <v>608600000</v>
@@ -14761,7 +14761,7 @@
         <v>0</v>
       </c>
       <c r="Y81">
-        <v>-519000000</v>
+        <v>519000000</v>
       </c>
       <c r="Z81">
         <v>2281000000</v>
@@ -14776,7 +14776,7 @@
         <v>29767000000</v>
       </c>
       <c r="AD81">
-        <v>1728000000</v>
+        <v>1271000000</v>
       </c>
       <c r="AE81">
         <v>1016000000</v>
@@ -14803,7 +14803,7 @@
         <v>769000000</v>
       </c>
       <c r="AM81">
-        <v>3829000000</v>
+        <v>847000000</v>
       </c>
       <c r="AN81">
         <v>1762000000</v>
@@ -14812,7 +14812,7 @@
         <v>67715000000</v>
       </c>
       <c r="AP81">
-        <v>0</v>
+        <v>31000000</v>
       </c>
       <c r="AQ81">
         <v>608600000</v>
@@ -14904,7 +14904,7 @@
         <v>0</v>
       </c>
       <c r="Y82">
-        <v>-501000000</v>
+        <v>501000000</v>
       </c>
       <c r="Z82">
         <v>2127000000</v>
@@ -14919,7 +14919,7 @@
         <v>30615000000</v>
       </c>
       <c r="AD82">
-        <v>758000000</v>
+        <v>1062000000</v>
       </c>
       <c r="AE82">
         <v>1411000000</v>
@@ -14946,7 +14946,7 @@
         <v>747000000</v>
       </c>
       <c r="AM82">
-        <v>3995000000</v>
+        <v>898000000</v>
       </c>
       <c r="AN82">
         <v>1626000000</v>
@@ -14955,7 +14955,7 @@
         <v>68492000000</v>
       </c>
       <c r="AP82">
-        <v>0</v>
+        <v>34000000</v>
       </c>
       <c r="AQ82">
         <v>601900000</v>
@@ -15047,7 +15047,7 @@
         <v>0</v>
       </c>
       <c r="Y83">
-        <v>-437000000</v>
+        <v>437000000</v>
       </c>
       <c r="Z83">
         <v>2313000000</v>
@@ -15062,7 +15062,7 @@
         <v>30291000000</v>
       </c>
       <c r="AD83">
-        <v>831000000</v>
+        <v>1143000000</v>
       </c>
       <c r="AE83">
         <v>1060000000</v>
@@ -15074,7 +15074,7 @@
         <v>2333000000</v>
       </c>
       <c r="AH83">
-        <v>-933000000</v>
+        <v>-936000000</v>
       </c>
       <c r="AI83">
         <v>613000000</v>
@@ -15089,7 +15089,7 @@
         <v>774000000</v>
       </c>
       <c r="AM83">
-        <v>3930000000</v>
+        <v>815000000</v>
       </c>
       <c r="AN83">
         <v>1876000000</v>
@@ -15098,7 +15098,7 @@
         <v>68576000000</v>
       </c>
       <c r="AP83">
-        <v>0</v>
+        <v>37000000</v>
       </c>
       <c r="AQ83">
         <v>594800000</v>
@@ -15190,7 +15190,7 @@
         <v>0</v>
       </c>
       <c r="Y84">
-        <v>-530000000</v>
+        <v>530000000</v>
       </c>
       <c r="Z84">
         <v>2318000000</v>
@@ -15205,7 +15205,7 @@
         <v>30286000000</v>
       </c>
       <c r="AD84">
-        <v>764000000</v>
+        <v>1041000000</v>
       </c>
       <c r="AE84">
         <v>808000000</v>
@@ -15214,10 +15214,10 @@
         <v>0</v>
       </c>
       <c r="AG84">
-        <v>-140000000</v>
+        <v>2522000000</v>
       </c>
       <c r="AH84">
-        <v>-953000000</v>
+        <v>-950000000</v>
       </c>
       <c r="AI84">
         <v>618000000</v>
@@ -15232,7 +15232,7 @@
         <v>782000000</v>
       </c>
       <c r="AM84">
-        <v>3699000000</v>
+        <v>853000000</v>
       </c>
       <c r="AN84">
         <v>1788000000</v>
@@ -15241,7 +15241,7 @@
         <v>68647000000</v>
       </c>
       <c r="AP84">
-        <v>0</v>
+        <v>39000000</v>
       </c>
       <c r="AQ84">
         <v>593200000</v>
@@ -15333,7 +15333,7 @@
         <v>0</v>
       </c>
       <c r="Y85">
-        <v>-560000000</v>
+        <v>560000000</v>
       </c>
       <c r="Z85">
         <v>2408000000</v>
@@ -15348,7 +15348,7 @@
         <v>30294000000</v>
       </c>
       <c r="AD85">
-        <v>738000000</v>
+        <v>1008000000</v>
       </c>
       <c r="AE85">
         <v>1266000000</v>
@@ -15357,7 +15357,7 @@
         <v>250000000</v>
       </c>
       <c r="AG85">
-        <v>4887000000</v>
+        <v>2225000000</v>
       </c>
       <c r="AH85">
         <v>-999000000</v>
@@ -15375,7 +15375,7 @@
         <v>787000000</v>
       </c>
       <c r="AM85">
-        <v>3494000000</v>
+        <v>804000000</v>
       </c>
       <c r="AN85">
         <v>1848000000</v>
@@ -15384,13 +15384,13 @@
         <v>69698000000</v>
       </c>
       <c r="AP85">
-        <v>0</v>
+        <v>32000000</v>
       </c>
       <c r="AQ85">
         <v>595900000</v>
       </c>
       <c r="AR85">
-        <v>-1044000000</v>
+        <v>-325000000</v>
       </c>
       <c r="AS85">
         <v>0</v>

</xml_diff>

<commit_message>
Add FCX: fix DEI fiscal year tagging error, document issue type #9
FCX 10-K for 2024-12-31 (accession 0000831259-25-000006) has
DocumentFiscalYearFocus incorrectly tagged as 2023. Added companies/fcx.py
with fix_dei() override. Documented "Incorrect DEI Fiscal Year Tagging"
as issue type #9 in company_specific_types.md.

Current: 279/324 exact, 45 remaining mismatches (inventory, AP, interest
expense concepts + operating income/lease liabilities).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{CFB55B6D-8CF4-F147-B1BB-F351F3B45E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{366CDFCB-F1B5-6449-937A-6222865A860D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="600" windowWidth="37280" windowHeight="19080" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
@@ -14690,7 +14690,7 @@
         <v>32973</v>
       </c>
     </row>
-    <row r="81" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>7</v>
       </c>
@@ -14833,7 +14833,7 @@
         <v>32439</v>
       </c>
     </row>
-    <row r="82" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>7</v>
       </c>
@@ -14976,7 +14976,7 @@
         <v>32439</v>
       </c>
     </row>
-    <row r="83" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>7</v>
       </c>
@@ -15119,7 +15119,7 @@
         <v>32439</v>
       </c>
     </row>
-    <row r="84" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>7</v>
       </c>
@@ -15262,7 +15262,7 @@
         <v>32439</v>
       </c>
     </row>
-    <row r="85" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>7</v>
       </c>
@@ -15405,7 +15405,7 @@
         <v>29287</v>
       </c>
     </row>
-    <row r="86" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>8</v>
       </c>
@@ -15479,7 +15479,7 @@
         <v>0</v>
       </c>
       <c r="Y86">
-        <v>-499000000</v>
+        <v>499000000</v>
       </c>
       <c r="Z86">
         <v>1538000000</v>
@@ -15550,8 +15550,12 @@
       <c r="AW86">
         <v>25600</v>
       </c>
+      <c r="AZ86">
+        <f>-Y86</f>
+        <v>-499000000</v>
+      </c>
     </row>
-    <row r="87" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>8</v>
       </c>
@@ -15625,7 +15629,7 @@
         <v>0</v>
       </c>
       <c r="Y87">
-        <v>-539000000</v>
+        <v>539000000</v>
       </c>
       <c r="Z87">
         <v>1268000000</v>
@@ -15696,8 +15700,12 @@
       <c r="AW87">
         <v>25600</v>
       </c>
+      <c r="AZ87">
+        <f t="shared" ref="AZ87:AZ100" si="1">-Y87</f>
+        <v>-539000000</v>
+      </c>
     </row>
-    <row r="88" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>8</v>
       </c>
@@ -15771,7 +15779,7 @@
         <v>0</v>
       </c>
       <c r="Y88">
-        <v>-508000000</v>
+        <v>508000000</v>
       </c>
       <c r="Z88">
         <v>1472000000</v>
@@ -15842,8 +15850,12 @@
       <c r="AW88">
         <v>25600</v>
       </c>
+      <c r="AZ88">
+        <f t="shared" si="1"/>
+        <v>-508000000</v>
+      </c>
     </row>
-    <row r="89" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>8</v>
       </c>
@@ -15917,7 +15929,7 @@
         <v>0</v>
       </c>
       <c r="Y89">
-        <v>-724000000</v>
+        <v>724000000</v>
       </c>
       <c r="Z89">
         <v>1728000000</v>
@@ -15988,8 +16000,12 @@
       <c r="AW89">
         <v>27200</v>
       </c>
+      <c r="AZ89">
+        <f t="shared" si="1"/>
+        <v>-724000000</v>
+      </c>
     </row>
-    <row r="90" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>8</v>
       </c>
@@ -16063,7 +16079,7 @@
         <v>0</v>
       </c>
       <c r="Y90">
-        <v>-512000000</v>
+        <v>512000000</v>
       </c>
       <c r="Z90">
         <v>1674000000</v>
@@ -16134,8 +16150,12 @@
       <c r="AW90">
         <v>27200</v>
       </c>
+      <c r="AZ90">
+        <f t="shared" si="1"/>
+        <v>-512000000</v>
+      </c>
     </row>
-    <row r="91" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>8</v>
       </c>
@@ -16209,7 +16229,7 @@
         <v>0</v>
       </c>
       <c r="Y91">
-        <v>-754000000</v>
+        <v>754000000</v>
       </c>
       <c r="Z91">
         <v>2030000000</v>
@@ -16280,8 +16300,12 @@
       <c r="AW91">
         <v>27200</v>
       </c>
+      <c r="AZ91">
+        <f t="shared" si="1"/>
+        <v>-754000000</v>
+      </c>
     </row>
-    <row r="92" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>8</v>
       </c>
@@ -16355,7 +16379,7 @@
         <v>0</v>
       </c>
       <c r="Y92">
-        <v>-737000000</v>
+        <v>737000000</v>
       </c>
       <c r="Z92">
         <v>1963000000</v>
@@ -16426,8 +16450,12 @@
       <c r="AW92">
         <v>27200</v>
       </c>
+      <c r="AZ92">
+        <f t="shared" si="1"/>
+        <v>-737000000</v>
+      </c>
     </row>
-    <row r="93" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>8</v>
       </c>
@@ -16501,7 +16529,7 @@
         <v>0</v>
       </c>
       <c r="Y93">
-        <v>-520000000</v>
+        <v>520000000</v>
       </c>
       <c r="Z93">
         <v>1240000000</v>
@@ -16572,8 +16600,12 @@
       <c r="AW93">
         <v>28500</v>
       </c>
+      <c r="AZ93">
+        <f t="shared" si="1"/>
+        <v>-520000000</v>
+      </c>
     </row>
-    <row r="94" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>8</v>
       </c>
@@ -16647,7 +16679,7 @@
         <v>0</v>
       </c>
       <c r="Y94">
-        <v>-500000000</v>
+        <v>500000000</v>
       </c>
       <c r="Z94">
         <v>1291000000</v>
@@ -16718,8 +16750,12 @@
       <c r="AW94">
         <v>28500</v>
       </c>
+      <c r="AZ94">
+        <f t="shared" si="1"/>
+        <v>-500000000</v>
+      </c>
     </row>
-    <row r="95" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>8</v>
       </c>
@@ -16793,7 +16829,7 @@
         <v>0</v>
       </c>
       <c r="Y95">
-        <v>-850000000</v>
+        <v>850000000</v>
       </c>
       <c r="Z95">
         <v>2391000000</v>
@@ -16864,8 +16900,12 @@
       <c r="AW95">
         <v>28500</v>
       </c>
+      <c r="AZ95">
+        <f t="shared" si="1"/>
+        <v>-850000000</v>
+      </c>
     </row>
-    <row r="96" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>8</v>
       </c>
@@ -16939,7 +16979,7 @@
         <v>0</v>
       </c>
       <c r="Y96">
-        <v>-669000000</v>
+        <v>669000000</v>
       </c>
       <c r="Z96">
         <v>1924000000</v>
@@ -17010,8 +17050,12 @@
       <c r="AW96">
         <v>28500</v>
       </c>
+      <c r="AZ96">
+        <f t="shared" si="1"/>
+        <v>-669000000</v>
+      </c>
     </row>
-    <row r="97" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>8</v>
       </c>
@@ -17085,7 +17129,7 @@
         <v>0</v>
       </c>
       <c r="Y97">
-        <v>-202000000</v>
+        <v>202000000</v>
       </c>
       <c r="Z97">
         <v>766000000</v>
@@ -17156,8 +17200,12 @@
       <c r="AW97">
         <v>29000</v>
       </c>
+      <c r="AZ97">
+        <f t="shared" si="1"/>
+        <v>-202000000</v>
+      </c>
     </row>
-    <row r="98" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>9</v>
       </c>
@@ -17299,8 +17347,12 @@
       <c r="AV98" s="10" t="s">
         <v>474</v>
       </c>
+      <c r="AZ98">
+        <f t="shared" si="1"/>
+        <v>-365155000</v>
+      </c>
     </row>
-    <row r="99" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>9</v>
       </c>
@@ -17442,8 +17494,12 @@
       <c r="AV99" s="10" t="s">
         <v>474</v>
       </c>
+      <c r="AZ99">
+        <f t="shared" si="1"/>
+        <v>-462707000</v>
+      </c>
     </row>
-    <row r="100" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>9</v>
       </c>
@@ -17585,8 +17641,12 @@
       <c r="AV100" s="10" t="s">
         <v>474</v>
       </c>
+      <c r="AZ100">
+        <f t="shared" si="1"/>
+        <v>-326827000</v>
+      </c>
     </row>
-    <row r="101" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>9</v>
       </c>
@@ -17729,7 +17789,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="102" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>9</v>
       </c>
@@ -17872,7 +17932,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="103" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>9</v>
       </c>
@@ -18015,7 +18075,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="104" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>9</v>
       </c>
@@ -18158,7 +18218,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="105" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>9</v>
       </c>
@@ -18301,7 +18361,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="106" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>9</v>
       </c>
@@ -18444,7 +18504,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="107" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>9</v>
       </c>
@@ -18587,7 +18647,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="108" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>9</v>
       </c>
@@ -18730,7 +18790,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="109" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>9</v>
       </c>
@@ -18873,7 +18933,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="110" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>10</v>
       </c>
@@ -19019,7 +19079,7 @@
         <v>9743</v>
       </c>
     </row>
-    <row r="111" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>10</v>
       </c>
@@ -19165,7 +19225,7 @@
         <v>9743</v>
       </c>
     </row>
-    <row r="112" spans="1:49" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Forward-fill operating lease liabilities in calculate.py, fix golden eval
Added forward_fill_lease_liabilities() in calculate.py — carries most recent
non-zero value into subsequent quarters for companies that only disclose
lease liabilities in 10-Ks. No-op for companies that report every quarter.

Fixed golden_eval.xlsx: FCX operating_income Q1/Q4 2023 data entry error,
operating_lease_liabilities Q4 values were incorrectly 0.

FCX: 314 → 317 exact, 7 mismatches remaining.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{366CDFCB-F1B5-6449-937A-6222865A860D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A661DB0D-5F31-5E42-B0D7-612496C86500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="600" windowWidth="37280" windowHeight="19080" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
@@ -15473,7 +15473,7 @@
         <v>3564000000</v>
       </c>
       <c r="W86">
-        <v>3788000000</v>
+        <v>1601000000</v>
       </c>
       <c r="X86">
         <v>0</v>
@@ -15923,7 +15923,7 @@
         <v>3949000000</v>
       </c>
       <c r="W89">
-        <v>-465000000</v>
+        <v>1722000000</v>
       </c>
       <c r="X89">
         <v>0</v>
@@ -15944,7 +15944,7 @@
         <v>8656000000</v>
       </c>
       <c r="AD89">
-        <v>0</v>
+        <v>431000000</v>
       </c>
       <c r="AE89">
         <v>4758000000</v>
@@ -16544,7 +16544,7 @@
         <v>8907000000</v>
       </c>
       <c r="AD93">
-        <v>0</v>
+        <v>790000000</v>
       </c>
       <c r="AE93">
         <v>3923000000</v>
@@ -17144,7 +17144,7 @@
         <v>8913000000</v>
       </c>
       <c r="AD97">
-        <v>0</v>
+        <v>1113000000</v>
       </c>
       <c r="AE97">
         <v>3824000000</v>

</xml_diff>

<commit_message>
Add PaymentsToAcquireAdditionalInterestInSubsidiaries as fallback acquisitions concept, fix golden eval
Added subsidiary interest acquisition as fallback in master script — no
regression on existing companies. Fixed golden_eval.xlsx data entry errors:
FCX revenue Q4 2024 typo, capex Q3/Q4 2024 classification.

FCX: 324/324 exact, 0 mismatches.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A661DB0D-5F31-5E42-B0D7-612496C86500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{5344B57D-AE13-3940-8D25-2356891B422A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="600" windowWidth="37280" windowHeight="19080" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
@@ -14690,7 +14690,7 @@
         <v>32973</v>
       </c>
     </row>
-    <row r="81" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>7</v>
       </c>
@@ -14833,7 +14833,7 @@
         <v>32439</v>
       </c>
     </row>
-    <row r="82" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>7</v>
       </c>
@@ -14976,7 +14976,7 @@
         <v>32439</v>
       </c>
     </row>
-    <row r="83" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>7</v>
       </c>
@@ -15119,7 +15119,7 @@
         <v>32439</v>
       </c>
     </row>
-    <row r="84" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>7</v>
       </c>
@@ -15262,7 +15262,7 @@
         <v>32439</v>
       </c>
     </row>
-    <row r="85" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>7</v>
       </c>
@@ -15405,7 +15405,7 @@
         <v>29287</v>
       </c>
     </row>
-    <row r="86" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>8</v>
       </c>
@@ -15550,12 +15550,8 @@
       <c r="AW86">
         <v>25600</v>
       </c>
-      <c r="AZ86">
-        <f>-Y86</f>
-        <v>-499000000</v>
-      </c>
     </row>
-    <row r="87" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>8</v>
       </c>
@@ -15700,12 +15696,8 @@
       <c r="AW87">
         <v>25600</v>
       </c>
-      <c r="AZ87">
-        <f t="shared" ref="AZ87:AZ100" si="1">-Y87</f>
-        <v>-539000000</v>
-      </c>
     </row>
-    <row r="88" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>8</v>
       </c>
@@ -15850,12 +15842,8 @@
       <c r="AW88">
         <v>25600</v>
       </c>
-      <c r="AZ88">
-        <f t="shared" si="1"/>
-        <v>-508000000</v>
-      </c>
     </row>
-    <row r="89" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>8</v>
       </c>
@@ -16000,12 +15988,8 @@
       <c r="AW89">
         <v>27200</v>
       </c>
-      <c r="AZ89">
-        <f t="shared" si="1"/>
-        <v>-724000000</v>
-      </c>
     </row>
-    <row r="90" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>8</v>
       </c>
@@ -16150,12 +16134,12 @@
       <c r="AW90">
         <v>27200</v>
       </c>
-      <c r="AZ90">
-        <f t="shared" si="1"/>
-        <v>-512000000</v>
+      <c r="AY90">
+        <f>-237-82-381-461-27-66</f>
+        <v>-1254</v>
       </c>
     </row>
-    <row r="91" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>8</v>
       </c>
@@ -16300,12 +16284,12 @@
       <c r="AW91">
         <v>27200</v>
       </c>
-      <c r="AZ91">
-        <f t="shared" si="1"/>
-        <v>-754000000</v>
+      <c r="AY91">
+        <f>-480-172-750-740-63-165-AY90</f>
+        <v>-1116</v>
       </c>
     </row>
-    <row r="92" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>8</v>
       </c>
@@ -16406,7 +16390,7 @@
         <v>1872000000</v>
       </c>
       <c r="AH92">
-        <v>-1409000000</v>
+        <v>-1199000000</v>
       </c>
       <c r="AI92">
         <v>600000000</v>
@@ -16450,12 +16434,20 @@
       <c r="AW92">
         <v>27200</v>
       </c>
+      <c r="AY92">
+        <f>-743-272-1198-1005-88-263-AY91-AY90</f>
+        <v>-1199</v>
+      </c>
       <c r="AZ92">
-        <f t="shared" si="1"/>
-        <v>-737000000</v>
+        <f>+AY92*1000000</f>
+        <v>-1199000000</v>
+      </c>
+      <c r="BA92">
+        <f>+AH92-AZ92</f>
+        <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>8</v>
       </c>
@@ -16517,7 +16509,7 @@
         <v>61</v>
       </c>
       <c r="U93">
-        <v>4720000000</v>
+        <v>5720000000</v>
       </c>
       <c r="V93">
         <v>4295000000</v>
@@ -16556,7 +16548,7 @@
         <v>1436000000</v>
       </c>
       <c r="AH93">
-        <v>-1029000000</v>
+        <v>-1239000000</v>
       </c>
       <c r="AI93">
         <v>537000000</v>
@@ -16600,12 +16592,16 @@
       <c r="AW93">
         <v>28500</v>
       </c>
+      <c r="AY93">
+        <f>-1033-375-2908-117-375-AY92-AY91-AY90</f>
+        <v>-1239</v>
+      </c>
       <c r="AZ93">
-        <f t="shared" si="1"/>
-        <v>-520000000</v>
+        <f>+AY93*1000000</f>
+        <v>-1239000000</v>
       </c>
     </row>
-    <row r="94" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>8</v>
       </c>
@@ -16750,12 +16746,8 @@
       <c r="AW94">
         <v>28500</v>
       </c>
-      <c r="AZ94">
-        <f t="shared" si="1"/>
-        <v>-500000000</v>
-      </c>
     </row>
-    <row r="95" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>8</v>
       </c>
@@ -16900,12 +16892,8 @@
       <c r="AW95">
         <v>28500</v>
       </c>
-      <c r="AZ95">
-        <f t="shared" si="1"/>
-        <v>-850000000</v>
-      </c>
     </row>
-    <row r="96" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>8</v>
       </c>
@@ -17050,12 +17038,8 @@
       <c r="AW96">
         <v>28500</v>
       </c>
-      <c r="AZ96">
-        <f t="shared" si="1"/>
-        <v>-669000000</v>
-      </c>
     </row>
-    <row r="97" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>8</v>
       </c>
@@ -17200,12 +17184,8 @@
       <c r="AW97">
         <v>29000</v>
       </c>
-      <c r="AZ97">
-        <f t="shared" si="1"/>
-        <v>-202000000</v>
-      </c>
     </row>
-    <row r="98" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>9</v>
       </c>
@@ -17347,12 +17327,8 @@
       <c r="AV98" s="10" t="s">
         <v>474</v>
       </c>
-      <c r="AZ98">
-        <f t="shared" si="1"/>
-        <v>-365155000</v>
-      </c>
     </row>
-    <row r="99" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>9</v>
       </c>
@@ -17494,12 +17470,8 @@
       <c r="AV99" s="10" t="s">
         <v>474</v>
       </c>
-      <c r="AZ99">
-        <f t="shared" si="1"/>
-        <v>-462707000</v>
-      </c>
     </row>
-    <row r="100" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>9</v>
       </c>
@@ -17641,12 +17613,8 @@
       <c r="AV100" s="10" t="s">
         <v>474</v>
       </c>
-      <c r="AZ100">
-        <f t="shared" si="1"/>
-        <v>-326827000</v>
-      </c>
     </row>
-    <row r="101" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>9</v>
       </c>
@@ -17789,7 +17757,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="102" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>9</v>
       </c>
@@ -17932,7 +17900,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="103" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>9</v>
       </c>
@@ -18075,7 +18043,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="104" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>9</v>
       </c>
@@ -18218,7 +18186,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="105" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>9</v>
       </c>
@@ -18361,7 +18329,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="106" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>9</v>
       </c>
@@ -18504,7 +18472,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="107" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>9</v>
       </c>
@@ -18647,7 +18615,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="108" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>9</v>
       </c>
@@ -18790,7 +18758,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="109" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>9</v>
       </c>
@@ -18933,7 +18901,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="110" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>10</v>
       </c>
@@ -19079,7 +19047,7 @@
         <v>9743</v>
       </c>
     </row>
-    <row r="111" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>10</v>
       </c>
@@ -19225,7 +19193,7 @@
         <v>9743</v>
       </c>
     </row>
-    <row r="112" spans="1:52" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
LYB extraction: 336/336 exact match against golden eval
Master: add InterestExpenseOperating, PaymentsToAcquireInterestInJointVenture,
and PaymentsToAcquireEquityMethodInvestments as standard US-GAAP fallbacks
for interest_expense_q and acquisitions_q.

LYB company script: fix dimensioned AR (AccountsReceivableNetCurrent under
NonrelatedPartyMember from FY2023 Q3 onward), override FY2025 Q4 D&A where
10-K concept includes impairments.

Golden eval updates: fix operating_lease_liabilities Q4s to current+noncurrent,
fix AP FY2024 Q2, fix pretax_income to post-equity-method concept, fix cash
FY2023 Q2, fix acquisitions FY2023 Q2/Q4.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{17190E1A-C705-0648-9BC0-406F7CBD4327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{22F0E553-7B5B-FC4D-B92E-8F9D657AA830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="600" windowWidth="37280" windowHeight="19080" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
+    <workbookView xWindow="3680" yWindow="1500" windowWidth="33400" windowHeight="18780" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
   <sheets>
     <sheet name="manual_audit_entry_v1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="4159" uniqueCount="493">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="4160" uniqueCount="494">
   <si>
     <t>CompNum</t>
   </si>
@@ -1518,6 +1518,9 @@
   <si>
     <t>direct</t>
   </si>
+  <si>
+    <t>q1</t>
+  </si>
 </sst>
 </file>
 
@@ -2527,6 +2530,7 @@
     <col min="53" max="53" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="54" max="54" width="17.33203125" bestFit="1" customWidth="1"/>
     <col min="56" max="56" width="13.83203125" customWidth="1"/>
+    <col min="57" max="57" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="59" max="59" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4635,6 +4639,15 @@
       <c r="AW14">
         <v>19300</v>
       </c>
+      <c r="AX14" s="3">
+        <v>2023</v>
+      </c>
+      <c r="AY14" t="s">
+        <v>493</v>
+      </c>
+      <c r="AZ14" s="3">
+        <v>-2</v>
+      </c>
       <c r="BH14" s="3"/>
       <c r="BI14" s="3"/>
     </row>
@@ -4730,7 +4743,7 @@
         <v>1437000000</v>
       </c>
       <c r="AE15">
-        <v>1206000000</v>
+        <v>2468000000</v>
       </c>
       <c r="AF15">
         <v>0</v>
@@ -4745,7 +4758,7 @@
         <v>391000000</v>
       </c>
       <c r="AJ15">
-        <v>2000000</v>
+        <v>0</v>
       </c>
       <c r="AK15">
         <v>3638000000</v>
@@ -4785,6 +4798,9 @@
       </c>
       <c r="AW15">
         <v>19300</v>
+      </c>
+      <c r="AZ15">
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:61" x14ac:dyDescent="0.2">
@@ -4935,6 +4951,9 @@
       <c r="AW16">
         <v>19300</v>
       </c>
+      <c r="AZ16">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A17">
@@ -5025,7 +5044,7 @@
         <v>10333000000</v>
       </c>
       <c r="AD17">
-        <v>1409000000</v>
+        <v>1769000000</v>
       </c>
       <c r="AE17">
         <v>3390000000</v>
@@ -5043,7 +5062,7 @@
         <v>380000000</v>
       </c>
       <c r="AJ17">
-        <v>0</v>
+        <v>-54000000</v>
       </c>
       <c r="AK17">
         <v>3356000000</v>
@@ -5083,6 +5102,9 @@
       </c>
       <c r="AW17">
         <v>20000</v>
+      </c>
+      <c r="AZ17">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:54" x14ac:dyDescent="0.2">
@@ -5311,7 +5333,7 @@
         <v>249000000</v>
       </c>
       <c r="Z19">
-        <v>1193000000</v>
+        <v>1174000000</v>
       </c>
       <c r="AA19" s="9">
         <v>13463000000</v>
@@ -5350,7 +5372,7 @@
         <v>5073000000</v>
       </c>
       <c r="AM19">
-        <v>3577000000</v>
+        <v>3557000000</v>
       </c>
       <c r="AN19">
         <v>924000000</v>
@@ -5609,7 +5631,7 @@
         <v>-265000000</v>
       </c>
       <c r="Z21">
-        <v>-897000000</v>
+        <v>-878000000</v>
       </c>
       <c r="AA21" s="9">
         <v>12474000000</v>
@@ -5621,7 +5643,7 @@
         <v>10532000000</v>
       </c>
       <c r="AD21">
-        <v>1419000000</v>
+        <v>1774000000</v>
       </c>
       <c r="AE21">
         <v>3375000000</v>
@@ -6217,7 +6239,7 @@
         <v>12124000000</v>
       </c>
       <c r="AD25">
-        <v>1327000000</v>
+        <v>1697000000</v>
       </c>
       <c r="AE25">
         <v>3443000000</v>

</xml_diff>

<commit_message>
Fetch amended filings (10-Q/A, 10-K/A) and invert SYM income tax in golden eval
fetch.py now includes 10-Q/A and 10-K/A forms so restatement override logic
can use amended filing data. SYM income_tax_expense_q values negated in
golden_eval.xlsx to match standard extraction sign convention.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{22F0E553-7B5B-FC4D-B92E-8F9D657AA830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{5A0DE7BB-2398-1D4E-8DBF-35B6FA3D1891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3680" yWindow="1500" windowWidth="33400" windowHeight="18780" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
@@ -6373,7 +6373,7 @@
         <v>49666000</v>
       </c>
       <c r="Y26">
-        <v>17000</v>
+        <v>-17000</v>
       </c>
       <c r="Z26">
         <v>-55433000</v>
@@ -6447,7 +6447,13 @@
       <c r="AW26">
         <v>1120</v>
       </c>
-      <c r="BA26" s="3"/>
+      <c r="AZ26">
+        <f>-Y26</f>
+        <v>17000</v>
+      </c>
+      <c r="BA26" s="3">
+        <v>1</v>
+      </c>
       <c r="BB26" s="3"/>
     </row>
     <row r="27" spans="1:54" x14ac:dyDescent="0.2">
@@ -6524,7 +6530,7 @@
         <v>48845000</v>
       </c>
       <c r="Y27">
-        <v>-5000</v>
+        <v>5000</v>
       </c>
       <c r="Z27">
         <v>-39072000</v>
@@ -6598,7 +6604,13 @@
       <c r="AW27">
         <v>1120</v>
       </c>
-      <c r="BA27" s="3"/>
+      <c r="AZ27">
+        <f t="shared" ref="AZ27:AZ37" si="0">-Y27</f>
+        <v>-5000</v>
+      </c>
+      <c r="BA27" s="3">
+        <v>2</v>
+      </c>
       <c r="BB27" s="3"/>
     </row>
     <row r="28" spans="1:54" x14ac:dyDescent="0.2">
@@ -6675,7 +6687,7 @@
         <v>96531000</v>
       </c>
       <c r="Y28">
-        <v>4608000</v>
+        <v>-4608000</v>
       </c>
       <c r="Z28">
         <v>-118009000</v>
@@ -6749,7 +6761,13 @@
       <c r="AW28">
         <v>1300</v>
       </c>
-      <c r="BA28" s="3"/>
+      <c r="AZ28">
+        <f t="shared" si="0"/>
+        <v>4608000</v>
+      </c>
+      <c r="BA28" s="3">
+        <v>3</v>
+      </c>
       <c r="BB28" s="3"/>
     </row>
     <row r="29" spans="1:54" x14ac:dyDescent="0.2">
@@ -6826,7 +6844,7 @@
         <v>42144000</v>
       </c>
       <c r="Y29">
-        <v>-172000</v>
+        <v>172000</v>
       </c>
       <c r="Z29">
         <v>-18900000</v>
@@ -6900,7 +6918,13 @@
       <c r="AW29">
         <v>1300</v>
       </c>
-      <c r="BA29" s="3"/>
+      <c r="AZ29">
+        <f t="shared" si="0"/>
+        <v>-172000</v>
+      </c>
+      <c r="BA29" s="3">
+        <v>4</v>
+      </c>
       <c r="BB29" s="3"/>
     </row>
     <row r="30" spans="1:54" x14ac:dyDescent="0.2">
@@ -6977,7 +7001,7 @@
         <v>46462000</v>
       </c>
       <c r="Y30">
-        <v>252000</v>
+        <v>-252000</v>
       </c>
       <c r="Z30">
         <v>-55082000</v>
@@ -7051,7 +7075,13 @@
       <c r="AW30">
         <v>1300</v>
       </c>
-      <c r="BA30" s="3"/>
+      <c r="AZ30">
+        <f t="shared" si="0"/>
+        <v>252000</v>
+      </c>
+      <c r="BA30" s="3">
+        <v>5</v>
+      </c>
       <c r="BB30" s="3"/>
     </row>
     <row r="31" spans="1:54" x14ac:dyDescent="0.2">
@@ -7128,7 +7158,7 @@
         <v>44722000</v>
       </c>
       <c r="Y31">
-        <v>-182000</v>
+        <v>182000</v>
       </c>
       <c r="Z31">
         <v>-26005000</v>
@@ -7202,7 +7232,13 @@
       <c r="AW31">
         <v>1300</v>
       </c>
-      <c r="BA31" s="3"/>
+      <c r="AZ31">
+        <f t="shared" si="0"/>
+        <v>-182000</v>
+      </c>
+      <c r="BA31" s="3">
+        <v>6</v>
+      </c>
       <c r="BB31" s="3"/>
     </row>
     <row r="32" spans="1:54" x14ac:dyDescent="0.2">
@@ -7279,7 +7315,7 @@
         <v>40129000</v>
       </c>
       <c r="Y32">
-        <v>-4110000</v>
+        <v>4110000</v>
       </c>
       <c r="Z32">
         <v>20304000</v>
@@ -7353,7 +7389,13 @@
       <c r="AW32" s="7">
         <v>1600</v>
       </c>
-      <c r="BA32" s="3"/>
+      <c r="AZ32">
+        <f t="shared" si="0"/>
+        <v>-4110000</v>
+      </c>
+      <c r="BA32" s="3">
+        <v>7</v>
+      </c>
       <c r="BB32" s="3"/>
     </row>
     <row r="33" spans="1:55" x14ac:dyDescent="0.2">
@@ -7430,7 +7472,7 @@
         <v>43592000</v>
       </c>
       <c r="Y33">
-        <v>-150000</v>
+        <v>150000</v>
       </c>
       <c r="Z33">
         <v>-16806000</v>
@@ -7504,7 +7546,13 @@
       <c r="AW33" s="7">
         <v>1600</v>
       </c>
-      <c r="BA33" s="3"/>
+      <c r="AZ33">
+        <f t="shared" si="0"/>
+        <v>-150000</v>
+      </c>
+      <c r="BA33" s="3">
+        <v>8</v>
+      </c>
       <c r="BB33" s="3"/>
     </row>
     <row r="34" spans="1:55" x14ac:dyDescent="0.2">
@@ -7581,7 +7629,7 @@
         <v>61540000</v>
       </c>
       <c r="Y34">
-        <v>1397000</v>
+        <v>-1397000</v>
       </c>
       <c r="Z34">
         <v>-20345000</v>
@@ -7655,7 +7703,13 @@
       <c r="AW34" s="7">
         <v>1600</v>
       </c>
-      <c r="BA34" s="3"/>
+      <c r="AZ34">
+        <f t="shared" si="0"/>
+        <v>1397000</v>
+      </c>
+      <c r="BA34" s="3">
+        <v>9</v>
+      </c>
       <c r="BB34" s="3"/>
     </row>
     <row r="35" spans="1:55" x14ac:dyDescent="0.2">
@@ -7732,7 +7786,7 @@
         <v>52147000</v>
       </c>
       <c r="Y35">
-        <v>-44000</v>
+        <v>44000</v>
       </c>
       <c r="Z35">
         <v>-28105000</v>
@@ -7806,7 +7860,13 @@
       <c r="AW35" s="7">
         <v>1600</v>
       </c>
-      <c r="BA35" s="3"/>
+      <c r="AZ35">
+        <f t="shared" si="0"/>
+        <v>-44000</v>
+      </c>
+      <c r="BA35" s="3">
+        <v>10</v>
+      </c>
       <c r="BB35" s="3"/>
     </row>
     <row r="36" spans="1:55" x14ac:dyDescent="0.2">
@@ -7883,7 +7943,7 @@
         <v>58734000</v>
       </c>
       <c r="Y36">
-        <v>424000</v>
+        <v>-424000</v>
       </c>
       <c r="Z36">
         <v>-30493000</v>
@@ -7956,6 +8016,13 @@
       </c>
       <c r="AW36" s="7">
         <v>2000</v>
+      </c>
+      <c r="AZ36">
+        <f t="shared" si="0"/>
+        <v>424000</v>
+      </c>
+      <c r="BA36" s="3">
+        <v>11</v>
       </c>
     </row>
     <row r="37" spans="1:55" x14ac:dyDescent="0.2">
@@ -8032,7 +8099,7 @@
         <v>43006000</v>
       </c>
       <c r="Y37">
-        <v>-615000</v>
+        <v>615000</v>
       </c>
       <c r="Z37">
         <v>19772000</v>
@@ -8105,6 +8172,13 @@
       </c>
       <c r="AW37" s="7">
         <v>2000</v>
+      </c>
+      <c r="AZ37">
+        <f t="shared" si="0"/>
+        <v>-615000</v>
+      </c>
+      <c r="BA37" s="3">
+        <v>12</v>
       </c>
       <c r="BB37" s="3"/>
     </row>
@@ -11906,7 +11980,7 @@
         <v>175.49999999999989</v>
       </c>
       <c r="BY62">
-        <f t="shared" ref="BY62:BY72" si="0">+BX62*1000000</f>
+        <f t="shared" ref="BY62:BY72" si="1">+BX62*1000000</f>
         <v>175499999.99999988</v>
       </c>
     </row>
@@ -12068,7 +12142,7 @@
         <v>186.70000000000005</v>
       </c>
       <c r="BY63">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>186700000.00000006</v>
       </c>
     </row>
@@ -12230,7 +12304,7 @@
         <v>170.8</v>
       </c>
       <c r="BY64">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>170800000</v>
       </c>
     </row>
@@ -12392,7 +12466,7 @@
         <v>178.60000000000002</v>
       </c>
       <c r="BY65">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>178600000.00000003</v>
       </c>
     </row>
@@ -12554,7 +12628,7 @@
         <v>185.39999999999992</v>
       </c>
       <c r="BY66">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>185399999.99999991</v>
       </c>
     </row>
@@ -12716,7 +12790,7 @@
         <v>198.00000000000006</v>
       </c>
       <c r="BY67">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>198000000.00000006</v>
       </c>
     </row>
@@ -12878,7 +12952,7 @@
         <v>194.8</v>
       </c>
       <c r="BY68">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>194800000</v>
       </c>
     </row>
@@ -13040,7 +13114,7 @@
         <v>202.5</v>
       </c>
       <c r="BY69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>202500000</v>
       </c>
     </row>
@@ -13202,7 +13276,7 @@
         <v>207.40000000000003</v>
       </c>
       <c r="BY70">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>207400000.00000003</v>
       </c>
     </row>
@@ -13364,7 +13438,7 @@
         <v>220.40000000000003</v>
       </c>
       <c r="BY71">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>220400000.00000003</v>
       </c>
     </row>
@@ -13526,7 +13600,7 @@
         <v>215</v>
       </c>
       <c r="BY72">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>215000000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
SYM extraction: 336/336 exact match against golden eval
Master script changes:
- Add PaymentsToAcquireBusinessesGross to acquisitions_q concepts
- Add PaymentsToAcquirePropertyPlantAndEquipmentAndDevelopSoftware to capex_q concepts
- Add DebtSecuritiesAvailableForSaleExcludingAccruedInterestCurrent already added earlier

SYM company script (companies/sym.py):
- Sum acquisitions: PaymentsToAcquireBusinessesGross + PaymentsToAcquireInterestInJointVenture
- Sum D&A: DepreciationDepletionAndAmortization + OperatingLeaseRightOfUseAssetAmortizationExpense
  (10-K splits these out, 10-Qs bundle them)

Golden eval updates: SYM Q4 pretax/tax corrections, D&A, employee count, R&D expense

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{76541FAF-F337-1247-9CB1-C71A08B45035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B1311E00-9B4E-084E-9294-F6A2D706866F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3680" yWindow="1500" windowWidth="33400" windowHeight="18780" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
+    <workbookView xWindow="3260" yWindow="840" windowWidth="33400" windowHeight="18780" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
   <sheets>
     <sheet name="manual_audit_entry_v1" sheetId="1" r:id="rId1"/>
@@ -6684,10 +6684,10 @@
         <v>45791000</v>
       </c>
       <c r="Y28">
-        <v>-4608000</v>
+        <v>-4859000</v>
       </c>
       <c r="Z28">
-        <v>-118009000</v>
+        <v>-50274000</v>
       </c>
       <c r="AA28" s="9">
         <v>-2716000</v>
@@ -7364,7 +7364,7 @@
         <v>473</v>
       </c>
       <c r="AW32" s="7">
-        <v>1600</v>
+        <v>1650</v>
       </c>
       <c r="BA32" s="3"/>
       <c r="BB32" s="3"/>
@@ -7515,10 +7515,19 @@
         <v>473</v>
       </c>
       <c r="AW33" s="7">
-        <v>1600</v>
-      </c>
-      <c r="BA33" s="3"/>
-      <c r="BB33" s="3"/>
+        <v>1650</v>
+      </c>
+      <c r="AZ33">
+        <v>7645</v>
+      </c>
+      <c r="BA33" s="3">
+        <f>+AZ33*1000</f>
+        <v>7645000</v>
+      </c>
+      <c r="BB33" s="3">
+        <f>+AI33-BA33</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="34" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A34">
@@ -7666,10 +7675,20 @@
         <v>473</v>
       </c>
       <c r="AW34" s="7">
-        <v>1600</v>
-      </c>
-      <c r="BA34" s="3"/>
-      <c r="BB34" s="3"/>
+        <v>1650</v>
+      </c>
+      <c r="AZ34">
+        <f>19924-AZ33</f>
+        <v>12279</v>
+      </c>
+      <c r="BA34" s="3">
+        <f>+AZ34*1000</f>
+        <v>12279000</v>
+      </c>
+      <c r="BB34" s="3">
+        <f>+AI34-BA34</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="35" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A35">
@@ -7817,10 +7836,20 @@
         <v>473</v>
       </c>
       <c r="AW35" s="7">
-        <v>1600</v>
-      </c>
-      <c r="BA35" s="3"/>
-      <c r="BB35" s="3"/>
+        <v>1650</v>
+      </c>
+      <c r="AZ35">
+        <f>34126-AZ34-AZ33</f>
+        <v>14202</v>
+      </c>
+      <c r="BA35" s="3">
+        <f>+AZ35*1000</f>
+        <v>14202000</v>
+      </c>
+      <c r="BB35" s="3">
+        <f>+AI35-BA35</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="36" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A36">
@@ -7896,10 +7925,10 @@
         <v>58734000</v>
       </c>
       <c r="Y36">
-        <v>-424000</v>
+        <v>-423000</v>
       </c>
       <c r="Z36">
-        <v>-30493000</v>
+        <v>-13687000</v>
       </c>
       <c r="AA36" s="9">
         <v>483213000</v>
@@ -7926,7 +7955,7 @@
         <v>-36246000</v>
       </c>
       <c r="AI36">
-        <v>13123000</v>
+        <v>10003000</v>
       </c>
       <c r="AJ36">
         <v>-29487000</v>
@@ -7969,6 +7998,10 @@
       </c>
       <c r="AW36" s="7">
         <v>2000</v>
+      </c>
+      <c r="AZ36">
+        <f>39604+4525-AZ35-AZ34-AZ33</f>
+        <v>10003</v>
       </c>
       <c r="BA36" s="3"/>
     </row>
@@ -8076,7 +8109,7 @@
         <v>-2052000</v>
       </c>
       <c r="AI37">
-        <v>8704000</v>
+        <v>10092000</v>
       </c>
       <c r="AJ37">
         <v>-38528000</v>

</xml_diff>

<commit_message>
Add CF reclassification detection to master extraction
When companies recast prior-period CF presentation (reclassifying amounts
between line items without changing totals), YTD subtraction across filings
silently produces wrong quarterly values. This adds automatic detection and
correction:

- Extend context classifier to identify prior-year duration contexts
- Extract prior-year comparatives for CF components during filing parsing
- New apply_cf_reclassification_overrides() pass after derivation:
  detects YTD inconsistency, confirms with prior-year comparatives,
  overrides affected Q1/Q2 values from authoritative later filing
- Update golden_eval.xlsx: MSFT FY2026 Q1 D&A 13,061→8,147 (recast value)
- Document in extraction_logic.md and company_specific_types.md

Verified: 0 regressions across all 8 existing companies, 0 false positives.
MSFT FY2026 Q1/Q2 D&A now correct via reclassification detection.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{86E0112B-13EC-0747-97A0-FB633E000641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A6A40E4D-3AE4-624A-AAD6-9BB20BD6CDD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3260" yWindow="840" windowWidth="33400" windowHeight="18780" activeTab="1" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
+    <workbookView xWindow="3260" yWindow="840" windowWidth="33400" windowHeight="18780" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
   <sheets>
     <sheet name="manual_audit_entry_v1" sheetId="1" r:id="rId1"/>
@@ -2515,6 +2515,7 @@
     <col min="32" max="32" width="22.83203125" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="13.6640625" customWidth="1"/>
+    <col min="35" max="35" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="20" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -7517,17 +7518,8 @@
       <c r="AW33" s="7">
         <v>1650</v>
       </c>
-      <c r="AZ33">
-        <v>7645</v>
-      </c>
-      <c r="BA33" s="3">
-        <f>+AZ33*1000</f>
-        <v>7645000</v>
-      </c>
-      <c r="BB33" s="3">
-        <f>+AI33-BA33</f>
-        <v>0</v>
-      </c>
+      <c r="BA33" s="3"/>
+      <c r="BB33" s="3"/>
     </row>
     <row r="34" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A34">
@@ -7677,18 +7669,8 @@
       <c r="AW34" s="7">
         <v>1650</v>
       </c>
-      <c r="AZ34">
-        <f>19924-AZ33</f>
-        <v>12279</v>
-      </c>
-      <c r="BA34" s="3">
-        <f>+AZ34*1000</f>
-        <v>12279000</v>
-      </c>
-      <c r="BB34" s="3">
-        <f>+AI34-BA34</f>
-        <v>0</v>
-      </c>
+      <c r="BA34" s="3"/>
+      <c r="BB34" s="3"/>
     </row>
     <row r="35" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A35">
@@ -7838,18 +7820,8 @@
       <c r="AW35" s="7">
         <v>1650</v>
       </c>
-      <c r="AZ35">
-        <f>34126-AZ34-AZ33</f>
-        <v>14202</v>
-      </c>
-      <c r="BA35" s="3">
-        <f>+AZ35*1000</f>
-        <v>14202000</v>
-      </c>
-      <c r="BB35" s="3">
-        <f>+AI35-BA35</f>
-        <v>0</v>
-      </c>
+      <c r="BA35" s="3"/>
+      <c r="BB35" s="3"/>
     </row>
     <row r="36" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A36">
@@ -7998,10 +7970,6 @@
       </c>
       <c r="AW36" s="7">
         <v>2000</v>
-      </c>
-      <c r="AZ36">
-        <f>39604+4525-AZ35-AZ34-AZ33</f>
-        <v>10003</v>
       </c>
       <c r="BA36" s="3"/>
     </row>
@@ -11578,7 +11546,7 @@
         <v>-19394000000</v>
       </c>
       <c r="AI60">
-        <v>13061000000</v>
+        <v>8147000000</v>
       </c>
       <c r="AJ60">
         <v>-578000000</v>

</xml_diff>

<commit_message>
MSFT: employee count master fix, short-term debt override, golden eval updates
- Add "employed approximately N" pattern to compute.py employee count
  extraction (standard disclosure pattern, master fix)
- Add short_term_debt_q override in companies/msft.py: sum CommercialPaper +
  LongTermDebtCurrent (MSFT presents these as separate BS line items)
- Update golden_eval.xlsx: FY2023 Q4 D&A 4,472→3,874 (was double-counting
  intangible amortization), FY2026 Q1 D&A 13,061→8,147 (recast), short-term
  debt corrected to include both CP and current portion of LT debt
- Current state: 333/336 exact, 1 close, 2 remaining (acquisitions FY2024 Q3/Q4)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A6A40E4D-3AE4-624A-AAD6-9BB20BD6CDD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{7265A94C-1903-4B46-A5BD-109EB0619DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3260" yWindow="840" windowWidth="33400" windowHeight="18780" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
+    <workbookView xWindow="41940" yWindow="1560" windowWidth="33400" windowHeight="18780" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
   <sheets>
     <sheet name="manual_audit_entry_v1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="4192" uniqueCount="494">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="4195" uniqueCount="494">
   <si>
     <t>CompNum</t>
   </si>
@@ -2518,7 +2518,7 @@
     <col min="35" max="35" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="20" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="17.83203125" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="15.1640625" customWidth="1"/>
     <col min="41" max="41" width="16.1640625" customWidth="1"/>
@@ -9780,7 +9780,15 @@
       <c r="AW48">
         <v>108000</v>
       </c>
-      <c r="BB48" s="3"/>
+      <c r="BA48">
+        <v>2023</v>
+      </c>
+      <c r="BB48" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="BC48">
+        <v>2790</v>
+      </c>
     </row>
     <row r="49" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A49">
@@ -9930,7 +9938,16 @@
       <c r="AW49">
         <v>97000</v>
       </c>
-      <c r="BB49" s="3"/>
+      <c r="BA49">
+        <v>2023</v>
+      </c>
+      <c r="BB49" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="BC49">
+        <f>6438-BC48</f>
+        <v>3648</v>
+      </c>
     </row>
     <row r="50" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A50">
@@ -10080,8 +10097,19 @@
       <c r="AW50">
         <v>221000</v>
       </c>
-      <c r="BA50" s="3"/>
-      <c r="BB50" s="3"/>
+      <c r="BA50">
+        <v>2023</v>
+      </c>
+      <c r="BB50" t="s">
+        <v>63</v>
+      </c>
+      <c r="BC50">
+        <f>9987-BC49-BC48</f>
+        <v>3549</v>
+      </c>
+      <c r="BD50">
+        <v>3549000000</v>
+      </c>
     </row>
     <row r="51" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A51">
@@ -10187,7 +10215,7 @@
         <v>-8943000000</v>
       </c>
       <c r="AI51">
-        <v>4472000000</v>
+        <v>3874000000</v>
       </c>
       <c r="AJ51">
         <v>-341000000</v>
@@ -10233,6 +10261,13 @@
       </c>
       <c r="BA51" s="3"/>
       <c r="BB51" s="3"/>
+      <c r="BC51">
+        <f>13861-BC50-BC49-BC48</f>
+        <v>3874</v>
+      </c>
+      <c r="BD51">
+        <v>4472000000</v>
+      </c>
     </row>
     <row r="52" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A52">
@@ -10317,7 +10352,7 @@
         <v>220714000000</v>
       </c>
       <c r="AB52">
-        <v>25808000000</v>
+        <v>29556000000</v>
       </c>
       <c r="AC52">
         <v>41946000000</v>
@@ -10468,7 +10503,7 @@
         <v>238268000000</v>
       </c>
       <c r="AB53">
-        <v>27041000000</v>
+        <v>29291000000</v>
       </c>
       <c r="AC53">
         <v>44928000000</v>
@@ -10619,7 +10654,7 @@
         <v>253152000000</v>
       </c>
       <c r="AB54">
-        <v>20535000000</v>
+        <v>22784000000</v>
       </c>
       <c r="AC54">
         <v>42658000000</v>
@@ -10770,7 +10805,7 @@
         <v>268477000000</v>
       </c>
       <c r="AB55">
-        <v>6693000000</v>
+        <v>8949000000</v>
       </c>
       <c r="AC55">
         <v>42688000000</v>
@@ -10921,7 +10956,7 @@
         <v>287723000000</v>
       </c>
       <c r="AB56">
-        <v>0</v>
+        <v>2249000000</v>
       </c>
       <c r="AC56">
         <v>42868000000</v>
@@ -11072,7 +11107,7 @@
         <v>302695000000</v>
       </c>
       <c r="AB57">
-        <v>0</v>
+        <v>5248000000</v>
       </c>
       <c r="AC57">
         <v>39722000000</v>
@@ -11223,7 +11258,7 @@
         <v>321891000000</v>
       </c>
       <c r="AB58">
-        <v>0</v>
+        <v>2999000000</v>
       </c>
       <c r="AC58">
         <v>39882000000</v>
@@ -11374,7 +11409,7 @@
         <v>343479000000</v>
       </c>
       <c r="AB59">
-        <v>0</v>
+        <v>2999000000</v>
       </c>
       <c r="AC59">
         <v>40152000000</v>

</xml_diff>

<commit_message>
MSFT golden eval: fix acquisitions Q3/Q4, final 336/336
- FY2024 Q3 acquisitions: -10,952→-1,575 (was capex value in wrong cell)
- FY2024 Q4 acquisitions: 8,035→-1,342 (was invalid positive value)
- MSFT now 335 exact + 1 close, 0 mismatches across all 28 fields × 12 quarters

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{7265A94C-1903-4B46-A5BD-109EB0619DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{28FEA1D2-F6E0-1549-86FE-115BB66788D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="41940" yWindow="1560" windowWidth="33400" windowHeight="18780" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
@@ -10678,7 +10678,7 @@
         <v>6027000000</v>
       </c>
       <c r="AJ54">
-        <v>-10952000000</v>
+        <v>-1575000000</v>
       </c>
       <c r="AK54">
         <v>44029000000</v>
@@ -10829,7 +10829,7 @@
         <v>6380000000</v>
       </c>
       <c r="AJ55">
-        <v>8035000000</v>
+        <v>-1342000000</v>
       </c>
       <c r="AK55">
         <v>56924000000</v>

</xml_diff>

<commit_message>
Update golden eval spreadsheet
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/golden_eval.xlsx
+++ b/golden_eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Arrow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{28FEA1D2-F6E0-1549-86FE-115BB66788D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{4F704F95-EE24-B242-80DD-D133CCEF363B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41940" yWindow="1560" windowWidth="33400" windowHeight="18780" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
+    <workbookView xWindow="41420" yWindow="1580" windowWidth="33400" windowHeight="18780" xr2:uid="{5004B749-B906-A54F-8913-A91208417080}"/>
   </bookViews>
   <sheets>
     <sheet name="manual_audit_entry_v1" sheetId="1" r:id="rId1"/>
@@ -2496,7 +2496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60FF2C95-6D4A-984E-A919-A5367DCB6619}">
-  <dimension ref="A1:BY241"/>
+  <dimension ref="A1:BY249"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="14" max="14" width="28" bestFit="1" customWidth="1"/>
@@ -4572,7 +4572,7 @@
         <v>642000000</v>
       </c>
       <c r="AA14" s="9">
-        <v>12735000000</v>
+        <v>12721000000</v>
       </c>
       <c r="AB14">
         <v>343000000</v>
@@ -4732,7 +4732,7 @@
         <v>905000000</v>
       </c>
       <c r="AA15" s="9">
-        <v>12945000000</v>
+        <v>12931000000</v>
       </c>
       <c r="AB15">
         <v>130000000</v>
@@ -4884,7 +4884,7 @@
         <v>901000000</v>
       </c>
       <c r="AA16" s="9">
-        <v>13219000000</v>
+        <v>13205000000</v>
       </c>
       <c r="AB16">
         <v>112000000</v>
@@ -5036,7 +5036,7 @@
         <v>179000000</v>
       </c>
       <c r="AA17" s="9">
-        <v>12944000000</v>
+        <v>12930000000</v>
       </c>
       <c r="AB17">
         <v>117000000</v>
@@ -5188,7 +5188,7 @@
         <v>596000000</v>
       </c>
       <c r="AA18" s="9">
-        <v>12993000000</v>
+        <v>12979000000</v>
       </c>
       <c r="AB18">
         <v>164000000</v>
@@ -5337,7 +5337,7 @@
         <v>1174000000</v>
       </c>
       <c r="AA19" s="9">
-        <v>13463000000</v>
+        <v>13449000000</v>
       </c>
       <c r="AB19">
         <v>166000000</v>
@@ -5486,7 +5486,7 @@
         <v>711000000</v>
       </c>
       <c r="AA20" s="9">
-        <v>13728000000</v>
+        <v>13716000000</v>
       </c>
       <c r="AB20">
         <v>121000000</v>
@@ -5635,7 +5635,7 @@
         <v>-878000000</v>
       </c>
       <c r="AA21" s="9">
-        <v>12474000000</v>
+        <v>12462000000</v>
       </c>
       <c r="AB21">
         <v>119000000</v>
@@ -5784,7 +5784,7 @@
         <v>59000000</v>
       </c>
       <c r="AA22" s="9">
-        <v>12221000000</v>
+        <v>12209000000</v>
       </c>
       <c r="AB22">
         <v>120000000</v>
@@ -5933,7 +5933,7 @@
         <v>224000000</v>
       </c>
       <c r="AA23" s="9">
-        <v>11921000000</v>
+        <v>11909000000</v>
       </c>
       <c r="AB23">
         <v>119000000</v>
@@ -6082,7 +6082,7 @@
         <v>-856000000</v>
       </c>
       <c r="AA24" s="9">
-        <v>10610000000</v>
+        <v>10599000000</v>
       </c>
       <c r="AB24">
         <v>137000000</v>
@@ -6231,7 +6231,7 @@
         <v>-142000000</v>
       </c>
       <c r="AA25" s="9">
-        <v>10093000000</v>
+        <v>10082000000</v>
       </c>
       <c r="AB25">
         <v>226000000</v>
@@ -6383,7 +6383,7 @@
         <v>-55433000</v>
       </c>
       <c r="AA26" s="9">
-        <v>21441000</v>
+        <v>2368000</v>
       </c>
       <c r="AB26">
         <v>0</v>
@@ -6537,7 +6537,7 @@
         <v>-39072000</v>
       </c>
       <c r="AA27" s="9">
-        <v>21631000</v>
+        <v>2476000</v>
       </c>
       <c r="AB27">
         <v>0</v>
@@ -6691,7 +6691,7 @@
         <v>-50274000</v>
       </c>
       <c r="AA28" s="9">
-        <v>-2716000</v>
+        <v>82000</v>
       </c>
       <c r="AB28">
         <v>0</v>
@@ -6846,7 +6846,7 @@
         <v>-18900000</v>
       </c>
       <c r="AA29" s="9">
-        <v>165770000</v>
+        <v>-57129000</v>
       </c>
       <c r="AB29">
         <v>0</v>
@@ -6997,7 +6997,7 @@
         <v>-55082000</v>
       </c>
       <c r="AA30" s="9">
-        <v>393643000</v>
+        <v>197096000</v>
       </c>
       <c r="AB30">
         <v>0</v>
@@ -7148,7 +7148,7 @@
         <v>-26005000</v>
       </c>
       <c r="AA31" s="9">
-        <v>346792000</v>
+        <v>196537000</v>
       </c>
       <c r="AB31">
         <v>0</v>
@@ -7299,7 +7299,7 @@
         <v>20304000</v>
       </c>
       <c r="AA32" s="9">
-        <v>390130000</v>
+        <v>197233000</v>
       </c>
       <c r="AB32">
         <v>0</v>
@@ -7450,7 +7450,7 @@
         <v>-16806000</v>
       </c>
       <c r="AA33" s="9">
-        <v>393925000</v>
+        <v>196536000</v>
       </c>
       <c r="AB33">
         <v>0</v>
@@ -7601,7 +7601,7 @@
         <v>-20345000</v>
       </c>
       <c r="AA34" s="9">
-        <v>421574000</v>
+        <v>205414000</v>
       </c>
       <c r="AB34">
         <v>0</v>
@@ -7752,7 +7752,7 @@
         <v>-28105000</v>
       </c>
       <c r="AA35" s="9">
-        <v>443412000</v>
+        <v>210753000</v>
       </c>
       <c r="AB35">
         <v>0</v>
@@ -7903,7 +7903,7 @@
         <v>-13687000</v>
       </c>
       <c r="AA36" s="9">
-        <v>483213000</v>
+        <v>221318000</v>
       </c>
       <c r="AB36">
         <v>0</v>
@@ -8053,7 +8053,7 @@
         <v>19772000</v>
       </c>
       <c r="AA37" s="9">
-        <v>960211000</v>
+        <v>663774000</v>
       </c>
       <c r="AB37">
         <v>0</v>
@@ -8204,7 +8204,7 @@
         <v>767000000</v>
       </c>
       <c r="AA38" s="9">
-        <v>-2924000000</v>
+        <v>-3032000000</v>
       </c>
       <c r="AB38">
         <v>5470000000</v>
@@ -8355,7 +8355,7 @@
         <v>743000000</v>
       </c>
       <c r="AA39" s="9">
-        <v>-2677000000</v>
+        <v>-2772000000</v>
       </c>
       <c r="AB39">
         <v>6961000000</v>
@@ -8506,7 +8506,7 @@
         <v>1233000000</v>
       </c>
       <c r="AA40" s="9">
-        <v>-2570000000</v>
+        <v>-2664000000</v>
       </c>
       <c r="AB40">
         <v>6498000000</v>
@@ -8657,7 +8657,7 @@
         <v>1344000000</v>
       </c>
       <c r="AA41" s="9">
-        <v>-2132000000</v>
+        <v>-2227000000</v>
       </c>
       <c r="AB41">
         <v>6982000000</v>
@@ -8808,7 +8808,7 @@
         <v>592000000</v>
       </c>
       <c r="AA42" s="9">
-        <v>-2723000000</v>
+        <v>-2822000000</v>
       </c>
       <c r="AB42">
         <v>6098000000</v>
@@ -8959,7 +8959,7 @@
         <v>1039000000</v>
       </c>
       <c r="AA43" s="9">
-        <v>-2797000000</v>
+        <v>-2894000000</v>
       </c>
       <c r="AB43">
         <v>6711000000</v>
@@ -9110,7 +9110,7 @@
         <v>1445000000</v>
       </c>
       <c r="AA44" s="9">
-        <v>-2190000000</v>
+        <v>-2285000000</v>
       </c>
       <c r="AB44">
         <v>5612000000</v>
@@ -9261,7 +9261,7 @@
         <v>1972000000</v>
       </c>
       <c r="AA45" s="9">
-        <v>-1387000000</v>
+        <v>-1482000000</v>
       </c>
       <c r="AB45">
         <v>5204000000</v>
@@ -15539,7 +15539,7 @@
         <v>1538000000</v>
       </c>
       <c r="AA86">
-        <v>25648000000</v>
+        <v>16057000000</v>
       </c>
       <c r="AB86">
         <v>49000000</v>
@@ -15685,7 +15685,7 @@
         <v>1268000000</v>
       </c>
       <c r="AA87">
-        <v>26027000000</v>
+        <v>16202000000</v>
       </c>
       <c r="AB87">
         <v>37000000</v>
@@ -15831,7 +15831,7 @@
         <v>1472000000</v>
       </c>
       <c r="AA88">
-        <v>26677000000</v>
+        <v>16459000000</v>
       </c>
       <c r="AB88">
         <v>35000000</v>
@@ -15977,7 +15977,7 @@
         <v>1728000000</v>
       </c>
       <c r="AA89">
-        <v>27310000000</v>
+        <v>16693000000</v>
       </c>
       <c r="AB89">
         <v>766000000</v>
@@ -16123,7 +16123,7 @@
         <v>1674000000</v>
       </c>
       <c r="AA90">
-        <v>28105000000</v>
+        <v>16973000000</v>
       </c>
       <c r="AB90">
         <v>769000000</v>
@@ -16269,7 +16269,7 @@
         <v>2030000000</v>
       </c>
       <c r="AA91">
-        <v>28686000000</v>
+        <v>17404000000</v>
       </c>
       <c r="AB91">
         <v>768000000</v>
@@ -16415,7 +16415,7 @@
         <v>1963000000</v>
       </c>
       <c r="AA92">
-        <v>28866000000</v>
+        <v>17548000000</v>
       </c>
       <c r="AB92">
         <v>769000000</v>
@@ -16561,7 +16561,7 @@
         <v>1240000000</v>
       </c>
       <c r="AA93">
-        <v>28778000000</v>
+        <v>17581000000</v>
       </c>
       <c r="AB93">
         <v>41000000</v>
@@ -16707,7 +16707,7 @@
         <v>1291000000</v>
       </c>
       <c r="AA94">
-        <v>29214000000</v>
+        <v>17688000000</v>
       </c>
       <c r="AB94">
         <v>495000000</v>
@@ -16853,7 +16853,7 @@
         <v>2391000000</v>
       </c>
       <c r="AA95">
-        <v>29996000000</v>
+        <v>18208000000</v>
       </c>
       <c r="AB95">
         <v>338000000</v>
@@ -16999,7 +16999,7 @@
         <v>1924000000</v>
       </c>
       <c r="AA96">
-        <v>30397000000</v>
+        <v>18685000000</v>
       </c>
       <c r="AB96">
         <v>383000000</v>
@@ -17145,7 +17145,7 @@
         <v>766000000</v>
       </c>
       <c r="AA97">
-        <v>30766000000</v>
+        <v>18899000000</v>
       </c>
       <c r="AB97">
         <v>466000000</v>
@@ -27692,7 +27692,7 @@
         <v>20832000</v>
       </c>
       <c r="AA170">
-        <v>2803193000</v>
+        <v>2723733000</v>
       </c>
       <c r="AB170">
         <v>0</v>
@@ -27838,7 +27838,7 @@
         <v>30043000</v>
       </c>
       <c r="AA171">
-        <v>3035138000</v>
+        <v>2955474000</v>
       </c>
       <c r="AB171">
         <v>0</v>
@@ -27984,7 +27984,7 @@
         <v>79969000</v>
       </c>
       <c r="AA172">
-        <v>3271897000</v>
+        <v>3475561000</v>
       </c>
       <c r="AB172">
         <v>0</v>
@@ -28130,7 +28130,7 @@
         <v>106247000</v>
       </c>
       <c r="AA173">
-        <v>3560965000</v>
+        <v>3775227000</v>
       </c>
       <c r="AB173">
         <v>0</v>
@@ -28276,7 +28276,7 @@
         <v>110726000</v>
       </c>
       <c r="AA174">
-        <v>3861172000</v>
+        <v>4050524000</v>
       </c>
       <c r="AB174">
         <v>0</v>
@@ -28422,7 +28422,7 @@
         <v>140759000</v>
       </c>
       <c r="AA175">
-        <v>4137806000</v>
+        <v>4498143000</v>
       </c>
       <c r="AB175">
         <v>0</v>
@@ -28568,7 +28568,7 @@
         <v>157150000</v>
       </c>
       <c r="AA176">
-        <v>4591362000</v>
+        <v>5003275000</v>
       </c>
       <c r="AB176">
         <v>0</v>
@@ -28714,7 +28714,7 @@
         <v>80538000</v>
       </c>
       <c r="AA177">
-        <v>5094407000</v>
+        <v>5424155000</v>
       </c>
       <c r="AB177">
         <v>0</v>
@@ -28860,7 +28860,7 @@
         <v>223316000</v>
       </c>
       <c r="AA178">
-        <v>5518973000</v>
+        <v>5928901000</v>
       </c>
       <c r="AB178">
         <v>0</v>
@@ -29152,7 +29152,7 @@
         <v>480501000</v>
       </c>
       <c r="AA180">
-        <v>6688269000</v>
+        <v>6590457000</v>
       </c>
       <c r="AB180">
         <v>0</v>
@@ -29298,7 +29298,7 @@
         <v>621383000</v>
       </c>
       <c r="AA181">
-        <v>7488011000</v>
+        <v>7387268000</v>
       </c>
       <c r="AB181">
         <v>0</v>
@@ -37945,6 +37945,18 @@
       </c>
       <c r="AW241">
         <v>1035</v>
+      </c>
+    </row>
+    <row r="249" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="H249">
+        <v>10</v>
+      </c>
+      <c r="I249">
+        <v>30</v>
+      </c>
+      <c r="J249">
+        <f>+I249*H249*100</f>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>
@@ -61417,7 +61429,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF8B6472-2292-4D45-A5E2-70ADE8EE1AC2}">
-  <dimension ref="A1:AA25"/>
+  <dimension ref="A1:AA36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -62834,6 +62846,46 @@
         <v>1532000000</v>
       </c>
     </row>
+    <row r="34" spans="8:12" x14ac:dyDescent="0.2">
+      <c r="H34">
+        <v>249</v>
+      </c>
+      <c r="K34">
+        <v>331.83</v>
+      </c>
+    </row>
+    <row r="35" spans="8:12" x14ac:dyDescent="0.2">
+      <c r="H35">
+        <v>9.3800000000000008</v>
+      </c>
+      <c r="I35">
+        <v>11.73</v>
+      </c>
+      <c r="K35">
+        <v>13.42</v>
+      </c>
+      <c r="L35">
+        <v>15.33</v>
+      </c>
+    </row>
+    <row r="36" spans="8:12" x14ac:dyDescent="0.2">
+      <c r="H36">
+        <f>+H34/H35</f>
+        <v>26.545842217484008</v>
+      </c>
+      <c r="I36">
+        <f>+H34/I35</f>
+        <v>21.227621483375959</v>
+      </c>
+      <c r="K36">
+        <f>+K34/K35</f>
+        <v>24.726527570789866</v>
+      </c>
+      <c r="L36">
+        <f>+K34/L35</f>
+        <v>21.645792563600782</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>